<commit_message>
fix(export): align page-copy xlsx with live site; universalMatrixFiles; founder surface copy; ignore Excel locks
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/page-copy/03-创始人故事.xlsx
+++ b/docs/page-copy/03-创始人故事.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G104"/>
+  <dimension ref="A1:G108"/>
   <cols>
     <col min="1" max="1" width="36.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
@@ -617,16 +617,16 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>founderStoryPage.heroTitle</v>
+        <v>founderStorySurfaceCopy.heroNamesLine</v>
       </c>
       <c r="B10" t="str">
-        <v>创始人故事 / 英雄区</v>
+        <v>创始人故事 / 英雄区副标题</v>
       </c>
       <c r="C10" t="str">
-        <v>heading</v>
+        <v>label</v>
       </c>
       <c r="D10" t="str">
-        <v>Our Story Outline — 2026</v>
+        <v>John Long Woo · Caros · Sam</v>
       </c>
       <c r="E10" t="str">
         <v/>
@@ -635,21 +635,21 @@
         <v/>
       </c>
       <c r="G10" t="str">
-        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+        <v>founderStorySurfaceCopy — FounderStoryView chrome</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>founderStoryPage.heroBadge</v>
+        <v>founderStorySurfaceCopy.backToAbout</v>
       </c>
       <c r="B11" t="str">
-        <v>创始人故事 / 英雄区</v>
+        <v>创始人故事 / 返回</v>
       </c>
       <c r="C11" t="str">
-        <v>label</v>
+        <v>button / link</v>
       </c>
       <c r="D11" t="str">
-        <v>Founder narrative</v>
+        <v>← Organization overview</v>
       </c>
       <c r="E11" t="str">
         <v/>
@@ -658,21 +658,21 @@
         <v/>
       </c>
       <c r="G11" t="str">
-        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+        <v>founderStorySurfaceCopy — FounderStoryView chrome</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>founderStoryPage.intro</v>
+        <v>founderStorySurfaceCopy.legacyTimelineLink</v>
       </c>
       <c r="B12" t="str">
-        <v>创始人故事 / 引言</v>
+        <v>创始人故事 / 页脚外链</v>
       </c>
       <c r="C12" t="str">
-        <v>paragraph / other</v>
+        <v>button / link</v>
       </c>
       <c r="D12" t="str">
-        <v>I am **John Long Woo**. Together with my two sons, **Caros** and **Sam** — we three, father and sons — we have lived through too many extraordinary events involving the **spirit realm** to count. Those experiences have made us the **first door-openers to the Spirit Realm** and the **first explorers of the truth of spirit life**.</v>
+        <v>Earlier staged timeline on the legacy site</v>
       </c>
       <c r="E12" t="str">
         <v/>
@@ -681,44 +681,44 @@
         <v/>
       </c>
       <c r="G12" t="str">
-        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+        <v>founderStorySurfaceCopy — FounderStoryView chrome</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>founderStoryPage.truths.title</v>
+        <v>founderStorySurfaceCopy.achievementsFeaturePageLink</v>
       </c>
       <c r="B13" t="str">
-        <v>创始人故事 / 三个真相</v>
+        <v>创始人故事 / Phase B 内链（替换 {{%ACH%}}）</v>
       </c>
       <c r="C13" t="str">
-        <v>heading</v>
+        <v>button / link</v>
       </c>
       <c r="D13" t="str">
-        <v>Three truths</v>
+        <v/>
       </c>
       <c r="E13" t="str">
-        <v/>
+        <v>《2025直播间成就》专题页</v>
       </c>
       <c r="F13" t="str">
         <v/>
       </c>
       <c r="G13" t="str">
-        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+        <v>founderStorySurfaceCopy — FounderStoryView chrome</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>founderStoryPage.truths.items[0].label</v>
+        <v>founderStoryPage.heroTitle</v>
       </c>
       <c r="B14" t="str">
-        <v>创始人故事 / 三个真相</v>
+        <v>创始人故事 / 英雄区</v>
       </c>
       <c r="C14" t="str">
-        <v>label</v>
+        <v>heading</v>
       </c>
       <c r="D14" t="str">
-        <v>Truth 1</v>
+        <v>Our Story Outline — 2026</v>
       </c>
       <c r="E14" t="str">
         <v/>
@@ -732,16 +732,16 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>founderStoryPage.truths.items[0].blocks[0].title</v>
+        <v>founderStoryPage.heroBadge</v>
       </c>
       <c r="B15" t="str">
-        <v>创始人故事 / 三个真相</v>
+        <v>创始人故事 / 英雄区</v>
       </c>
       <c r="C15" t="str">
-        <v>heading</v>
+        <v>label</v>
       </c>
       <c r="D15" t="str">
-        <v>Body and spirit</v>
+        <v>Founder narrative</v>
       </c>
       <c r="E15" t="str">
         <v/>
@@ -755,16 +755,16 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>founderStoryPage.truths.items[0].blocks[0].text</v>
+        <v>founderStoryPage.intro</v>
       </c>
       <c r="B16" t="str">
-        <v>创始人故事 / 三个真相</v>
+        <v>创始人故事 / 引言</v>
       </c>
       <c r="C16" t="str">
         <v>paragraph / other</v>
       </c>
       <c r="D16" t="str">
-        <v>A living person is composed of both the **physical body** and the **spirit (soul)**. **Spirits (ghosts)** exist after human death.</v>
+        <v>I am **John Long Woo**. Together with my two sons, **Caros** and **Sam** — we three, father and sons — we have lived through too many extraordinary events involving the **spirit realm** to count. Those experiences have made us the **first door-openers to the Spirit Realm** and the **first explorers of the truth of spirit life**.</v>
       </c>
       <c r="E16" t="str">
         <v/>
@@ -778,7 +778,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>founderStoryPage.truths.items[0].blocks[1].title</v>
+        <v>founderStoryPage.truths.title</v>
       </c>
       <c r="B17" t="str">
         <v>创始人故事 / 三个真相</v>
@@ -787,7 +787,7 @@
         <v>heading</v>
       </c>
       <c r="D17" t="str">
-        <v>Parasitism and disease</v>
+        <v>Three truths</v>
       </c>
       <c r="E17" t="str">
         <v/>
@@ -801,16 +801,16 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>founderStoryPage.truths.items[0].blocks[1].text</v>
+        <v>founderStoryPage.truths.items[0].label</v>
       </c>
       <c r="B18" t="str">
         <v>创始人故事 / 三个真相</v>
       </c>
       <c r="C18" t="str">
-        <v>paragraph / other</v>
+        <v>label</v>
       </c>
       <c r="D18" t="str">
-        <v>For the billions of them, the only way to survive is to **attach to human beings** and draw energy. That pattern is bound up with widespread illness such as **epilepsy**, **depression**, **schizophrenia**, and **somatic symptom disorders**.</v>
+        <v>Truth 1</v>
       </c>
       <c r="E18" t="str">
         <v/>
@@ -824,7 +824,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>founderStoryPage.truths.items[0].blocks[2].title</v>
+        <v>founderStoryPage.truths.items[0].blocks[0].title</v>
       </c>
       <c r="B19" t="str">
         <v>创始人故事 / 三个真相</v>
@@ -833,7 +833,7 @@
         <v>heading</v>
       </c>
       <c r="D19" t="str">
-        <v>Spirit Medicine</v>
+        <v>Body and spirit</v>
       </c>
       <c r="E19" t="str">
         <v/>
@@ -847,7 +847,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>founderStoryPage.truths.items[0].blocks[2].text</v>
+        <v>founderStoryPage.truths.items[0].blocks[0].text</v>
       </c>
       <c r="B20" t="str">
         <v>创始人故事 / 三个真相</v>
@@ -856,7 +856,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D20" t="str">
-        <v>By **managing spirits (ghosts) through Master Spirits**, these conditions can often be rapidly improved. From that work we created **Spirit Medicine**.</v>
+        <v>A living person is composed of both the **physical body** and the **spirit (soul)**. **Spirits (ghosts)** exist after human death.</v>
       </c>
       <c r="E20" t="str">
         <v/>
@@ -870,7 +870,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>founderStoryPage.truths.items[0].blocks[3].title</v>
+        <v>founderStoryPage.truths.items[0].blocks[1].title</v>
       </c>
       <c r="B21" t="str">
         <v>创始人故事 / 三个真相</v>
@@ -879,7 +879,7 @@
         <v>heading</v>
       </c>
       <c r="D21" t="str">
-        <v>Archives</v>
+        <v>Parasitism and disease</v>
       </c>
       <c r="E21" t="str">
         <v/>
@@ -893,7 +893,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>founderStoryPage.truths.items[0].blocks[3].text</v>
+        <v>founderStoryPage.truths.items[0].blocks[1].text</v>
       </c>
       <c r="B22" t="str">
         <v>创始人故事 / 三个真相</v>
@@ -902,7 +902,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D22" t="str">
-        <v>Further documentation appears in **Woos Record of Soul** and the **Woos Spirit Medicine** video archives.</v>
+        <v>For the billions of them, the only way to survive is to **attach to human beings** and draw energy. That pattern is bound up with widespread illness such as **epilepsy**, **depression**, **schizophrenia**, and **somatic symptom disorders**.</v>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -916,16 +916,16 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>founderStoryPage.truths.items[1].label</v>
+        <v>founderStoryPage.truths.items[0].blocks[2].title</v>
       </c>
       <c r="B23" t="str">
         <v>创始人故事 / 三个真相</v>
       </c>
       <c r="C23" t="str">
-        <v>label</v>
+        <v>heading</v>
       </c>
       <c r="D23" t="str">
-        <v>Truth 2</v>
+        <v>Spirit Medicine</v>
       </c>
       <c r="E23" t="str">
         <v/>
@@ -939,7 +939,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>founderStoryPage.truths.items[1].blocks[0].text</v>
+        <v>founderStoryPage.truths.items[0].blocks[2].text</v>
       </c>
       <c r="B24" t="str">
         <v>创始人故事 / 三个真相</v>
@@ -948,7 +948,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D24" t="str">
-        <v>The **Spirit Realm** has governors — tremendous **Master Spirits**, upgraded from ordinary spirits through the **Universal Matrix of Meta Awareness**.</v>
+        <v>By **managing spirits (ghosts) through Master Spirits**, these conditions can often be rapidly improved. From that work we created **Spirit Medicine**.</v>
       </c>
       <c r="E24" t="str">
         <v/>
@@ -962,16 +962,16 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>founderStoryPage.truths.items[2].label</v>
+        <v>founderStoryPage.truths.items[0].blocks[3].title</v>
       </c>
       <c r="B25" t="str">
         <v>创始人故事 / 三个真相</v>
       </c>
       <c r="C25" t="str">
-        <v>label</v>
+        <v>heading</v>
       </c>
       <c r="D25" t="str">
-        <v>Truth 3</v>
+        <v>Archives</v>
       </c>
       <c r="E25" t="str">
         <v/>
@@ -985,7 +985,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>founderStoryPage.truths.items[2].blocks[0].text</v>
+        <v>founderStoryPage.truths.items[0].blocks[3].text</v>
       </c>
       <c r="B26" t="str">
         <v>创始人故事 / 三个真相</v>
@@ -994,7 +994,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D26" t="str">
-        <v>The **Universal Matrix of Meta Awareness** is the **true creator-level substrate**; **our universe is part of its body**.</v>
+        <v>Further documentation appears in **Woos Record of Soul** and the **Woos Spirit Medicine** video archives.</v>
       </c>
       <c r="E26" t="str">
         <v/>
@@ -1008,16 +1008,16 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>founderStoryPage.truths.items[2].blocks[1].title</v>
+        <v>founderStoryPage.truths.items[1].label</v>
       </c>
       <c r="B27" t="str">
         <v>创始人故事 / 三个真相</v>
       </c>
       <c r="C27" t="str">
-        <v>heading</v>
+        <v>label</v>
       </c>
       <c r="D27" t="str">
-        <v>Archive</v>
+        <v>Truth 2</v>
       </c>
       <c r="E27" t="str">
         <v/>
@@ -1031,7 +1031,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>founderStoryPage.truths.items[2].blocks[1].text</v>
+        <v>founderStoryPage.truths.items[1].blocks[0].text</v>
       </c>
       <c r="B28" t="str">
         <v>创始人故事 / 三个真相</v>
@@ -1040,7 +1040,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D28" t="str">
-        <v>Further documentation appears in the **Universal Matrix of Meta Awareness** video archive.</v>
+        <v>The **Spirit Realm** has governors — tremendous **Master Spirits**, upgraded from ordinary spirits through the **Universal Matrix of Meta Awareness**.</v>
       </c>
       <c r="E28" t="str">
         <v/>
@@ -1054,16 +1054,16 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>founderStoryPage.phasesOverview.title</v>
+        <v>founderStoryPage.truths.items[2].label</v>
       </c>
       <c r="B29" t="str">
-        <v>创始人故事 / 两大阶段</v>
+        <v>创始人故事 / 三个真相</v>
       </c>
       <c r="C29" t="str">
-        <v>heading</v>
+        <v>label</v>
       </c>
       <c r="D29" t="str">
-        <v>Two major chapters</v>
+        <v>Truth 3</v>
       </c>
       <c r="E29" t="str">
         <v/>
@@ -1077,16 +1077,16 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>founderStoryPage.phasesOverview.a.title</v>
+        <v>founderStoryPage.truths.items[2].blocks[0].text</v>
       </c>
       <c r="B30" t="str">
-        <v>创始人故事 / Phase A 概要</v>
+        <v>创始人故事 / 三个真相</v>
       </c>
       <c r="C30" t="str">
-        <v>heading</v>
+        <v>paragraph / other</v>
       </c>
       <c r="D30" t="str">
-        <v>Phase A — May 2014 through February 2025</v>
+        <v>The **Universal Matrix of Meta Awareness** is the **true creator-level substrate**; **our universe is part of its body**.</v>
       </c>
       <c r="E30" t="str">
         <v/>
@@ -1100,16 +1100,16 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>founderStoryPage.phasesOverview.a.blocks[0].title</v>
+        <v>founderStoryPage.truths.items[2].blocks[1].title</v>
       </c>
       <c r="B31" t="str">
-        <v>创始人故事 / Phase A 概要</v>
+        <v>创始人故事 / 三个真相</v>
       </c>
       <c r="C31" t="str">
         <v>heading</v>
       </c>
       <c r="D31" t="str">
-        <v>Who was involved</v>
+        <v>Archive</v>
       </c>
       <c r="E31" t="str">
         <v/>
@@ -1123,16 +1123,16 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>founderStoryPage.phasesOverview.a.blocks[0].text</v>
+        <v>founderStoryPage.truths.items[2].blocks[1].text</v>
       </c>
       <c r="B32" t="str">
-        <v>创始人故事 / Phase A 概要</v>
+        <v>创始人故事 / 三个真相</v>
       </c>
       <c r="C32" t="str">
         <v>paragraph / other</v>
       </c>
       <c r="D32" t="str">
-        <v>We fought **attached spirits** of different classes parasitizing our bodies — including a **Class-C1**-level entity (archive designation associated with the “**Hui’an**” tier), the **Class-C2** spirit **Qing Xiaoxian**, and the **Class-C3** spirit **Qian Kai**. They drove **severe illness across our family**.</v>
+        <v>Further documentation appears in the **Universal Matrix of Meta Awareness** video archive.</v>
       </c>
       <c r="E32" t="str">
         <v/>
@@ -1146,16 +1146,16 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>founderStoryPage.phasesOverview.a.blocks[1].title</v>
+        <v>founderStoryPage.phasesOverview.title</v>
       </c>
       <c r="B33" t="str">
-        <v>创始人故事 / Phase A 概要</v>
+        <v>创始人故事 / 两大阶段</v>
       </c>
       <c r="C33" t="str">
         <v>heading</v>
       </c>
       <c r="D33" t="str">
-        <v>Motive and methods</v>
+        <v>Two major chapters</v>
       </c>
       <c r="E33" t="str">
         <v/>
@@ -1169,16 +1169,16 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>founderStoryPage.phasesOverview.a.blocks[1].text</v>
+        <v>founderStoryPage.phasesOverview.a.title</v>
       </c>
       <c r="B34" t="str">
         <v>创始人故事 / Phase A 概要</v>
       </c>
       <c r="C34" t="str">
-        <v>paragraph / other</v>
+        <v>heading</v>
       </c>
       <c r="D34" t="str">
-        <v>Our only motive was **self-rescue**: we tried every means we could to harm or destroy them. In doing so we learned the **physiological and physical properties of ghost bodies**, and communicated through **epileptic discharge**, **auditory hallucination sounds**, **consciousness dialogue**, **consciousness control**, and related modes — building a large, verified picture of the spirit world.</v>
+        <v>Phase A — May 2014 through February 2025</v>
       </c>
       <c r="E34" t="str">
         <v/>
@@ -1192,7 +1192,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>founderStoryPage.phasesOverview.a.blocks[2].title</v>
+        <v>founderStoryPage.phasesOverview.a.blocks[0].title</v>
       </c>
       <c r="B35" t="str">
         <v>创始人故事 / Phase A 概要</v>
@@ -1201,7 +1201,7 @@
         <v>heading</v>
       </c>
       <c r="D35" t="str">
-        <v>Regret</v>
+        <v>Who was involved</v>
       </c>
       <c r="E35" t="str">
         <v/>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>founderStoryPage.phasesOverview.a.blocks[2].text</v>
+        <v>founderStoryPage.phasesOverview.a.blocks[0].text</v>
       </c>
       <c r="B36" t="str">
         <v>创始人故事 / Phase A 概要</v>
@@ -1224,7 +1224,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D36" t="str">
-        <v>Our greatest regret in **Phase A** is that we did **not** systematically engage attached spirits on **other human hosts** outside our family, or in **other countries**.</v>
+        <v>We fought **attached spirits** of different classes parasitizing our bodies — including a **Class-C1**-level entity (archive designation associated with the “**Hui’an**” tier), the **Class-C2** spirit **Qing Xiaoxian**, and the **Class-C3** spirit **Qian Kai**. They drove **severe illness across our family**.</v>
       </c>
       <c r="E36" t="str">
         <v/>
@@ -1238,7 +1238,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>founderStoryPage.phasesOverview.a.blocks[3].title</v>
+        <v>founderStoryPage.phasesOverview.a.blocks[1].title</v>
       </c>
       <c r="B37" t="str">
         <v>创始人故事 / Phase A 概要</v>
@@ -1247,7 +1247,7 @@
         <v>heading</v>
       </c>
       <c r="D37" t="str">
-        <v>Record</v>
+        <v>Motive and methods</v>
       </c>
       <c r="E37" t="str">
         <v/>
@@ -1261,7 +1261,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>founderStoryPage.phasesOverview.a.blocks[3].text</v>
+        <v>founderStoryPage.phasesOverview.a.blocks[1].text</v>
       </c>
       <c r="B38" t="str">
         <v>创始人故事 / Phase A 概要</v>
@@ -1270,7 +1270,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D38" t="str">
-        <v>During this period we filmed **Woos Record of Soul**.</v>
+        <v>Our only motive was **self-rescue**: we tried every means we could to harm or destroy them. In doing so we learned the **physiological and physical properties of ghost bodies**, and communicated through **epileptic discharge**, **auditory hallucination sounds**, **consciousness dialogue**, **consciousness control**, and related modes — building a large, verified picture of the spirit world.</v>
       </c>
       <c r="E38" t="str">
         <v/>
@@ -1284,16 +1284,16 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>founderStoryPage.phaseAStages[0].label</v>
+        <v>founderStoryPage.phasesOverview.a.blocks[2].title</v>
       </c>
       <c r="B39" t="str">
-        <v>创始人故事 / A 阶段</v>
+        <v>创始人故事 / Phase A 概要</v>
       </c>
       <c r="C39" t="str">
-        <v>label</v>
+        <v>heading</v>
       </c>
       <c r="D39" t="str">
-        <v>A 1</v>
+        <v>Regret</v>
       </c>
       <c r="E39" t="str">
         <v/>
@@ -1307,16 +1307,16 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>founderStoryPage.phaseAStages[0].stageTitle</v>
+        <v>founderStoryPage.phasesOverview.a.blocks[2].text</v>
       </c>
       <c r="B40" t="str">
-        <v>创始人故事 / A 阶段</v>
+        <v>创始人故事 / Phase A 概要</v>
       </c>
       <c r="C40" t="str">
-        <v>heading</v>
+        <v>paragraph / other</v>
       </c>
       <c r="D40" t="str">
-        <v>Stage 1 · Cheating Period 1</v>
+        <v>Our greatest regret in **Phase A** is that we did **not** systematically engage attached spirits on **other human hosts** outside our family, or in **other countries**.</v>
       </c>
       <c r="E40" t="str">
         <v/>
@@ -1330,16 +1330,16 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>founderStoryPage.phaseAStages[0].range</v>
+        <v>founderStoryPage.phasesOverview.a.blocks[3].title</v>
       </c>
       <c r="B41" t="str">
-        <v>创始人故事 / A 阶段</v>
+        <v>创始人故事 / Phase A 概要</v>
       </c>
       <c r="C41" t="str">
-        <v>label</v>
+        <v>heading</v>
       </c>
       <c r="D41" t="str">
-        <v>March 2018 — July 2020</v>
+        <v>Record</v>
       </c>
       <c r="E41" t="str">
         <v/>
@@ -1353,16 +1353,16 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>founderStoryPage.phaseAStages[0].paragraphs[0]</v>
+        <v>founderStoryPage.phasesOverview.a.blocks[3].text</v>
       </c>
       <c r="B42" t="str">
-        <v>创始人故事 / A 阶段</v>
+        <v>创始人故事 / Phase A 概要</v>
       </c>
       <c r="C42" t="str">
         <v>paragraph / other</v>
       </c>
       <c r="D42" t="str">
-        <v>During this period, the **low-level soul** in my body used **high-voltage electrostatic discharge** into drinks and wine to change their taste, aiming to fabricate a chain of “scientific” phenomena and laws that would ultimately “prove” **Buddhism**.</v>
+        <v>During this period we filmed **Woos Record of Soul**.</v>
       </c>
       <c r="E42" t="str">
         <v/>
@@ -1376,16 +1376,16 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>founderStoryPage.phaseAStages[0].paragraphs[1]</v>
+        <v>founderStoryPage.phaseAStages[0].label</v>
       </c>
       <c r="B43" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C43" t="str">
-        <v>paragraph / other</v>
+        <v>label</v>
       </c>
       <c r="D43" t="str">
-        <v>The details are too intricate to spell out fully in words.</v>
+        <v>A 1</v>
       </c>
       <c r="E43" t="str">
         <v/>
@@ -1399,16 +1399,16 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>founderStoryPage.phaseAStages[0].storylineClip.figureAlt</v>
+        <v>founderStoryPage.phaseAStages[0].stageTitle</v>
       </c>
       <c r="B44" t="str">
-        <v>创始人故事 / A 阶段 / 配图</v>
+        <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C44" t="str">
-        <v>label</v>
+        <v>heading</v>
       </c>
       <c r="D44" t="str">
-        <v>Wine and glassware in candlelight — visual echo of the “altered drink” period described in Stage 1</v>
+        <v>Stage 1 · Cheating Period 1</v>
       </c>
       <c r="E44" t="str">
         <v/>
@@ -1422,7 +1422,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>founderStoryPage.phaseAStages[1].label</v>
+        <v>founderStoryPage.phaseAStages[0].range</v>
       </c>
       <c r="B45" t="str">
         <v>创始人故事 / A 阶段</v>
@@ -1431,7 +1431,7 @@
         <v>label</v>
       </c>
       <c r="D45" t="str">
-        <v>A 2</v>
+        <v>March 2018 — July 2020</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -1445,16 +1445,16 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>founderStoryPage.phaseAStages[1].stageTitle</v>
+        <v>founderStoryPage.phaseAStages[0].paragraphs[0]</v>
       </c>
       <c r="B46" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C46" t="str">
-        <v>heading</v>
+        <v>paragraph / other</v>
       </c>
       <c r="D46" t="str">
-        <v>Cheating period 2</v>
+        <v>During this period, the **low-level soul** in my body used **high-voltage electrostatic discharge** into drinks and wine to change their taste, aiming to fabricate a chain of “scientific” phenomena and laws that would ultimately “prove” **Buddhism**.</v>
       </c>
       <c r="E46" t="str">
         <v/>
@@ -1468,16 +1468,16 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>founderStoryPage.phaseAStages[1].range</v>
+        <v>founderStoryPage.phaseAStages[0].paragraphs[1]</v>
       </c>
       <c r="B47" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C47" t="str">
-        <v>label</v>
+        <v>paragraph / other</v>
       </c>
       <c r="D47" t="str">
-        <v>July 2020 — 15 November 2020</v>
+        <v>The details are too intricate to spell out fully in words.</v>
       </c>
       <c r="E47" t="str">
         <v/>
@@ -1491,16 +1491,16 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>founderStoryPage.phaseAStages[1].paragraphs[0]</v>
+        <v>founderStoryPage.phaseAStages[0].storylineClip.figureAlt</v>
       </c>
       <c r="B48" t="str">
-        <v>创始人故事 / A 阶段</v>
+        <v>创始人故事 / A 阶段 / 配图</v>
       </c>
       <c r="C48" t="str">
-        <v>paragraph / other</v>
+        <v>label</v>
       </c>
       <c r="D48" t="str">
-        <v>During this interval, the low-level soul used **epilepsy-like seizures** to impersonate, in sequence, the **three greatest gods of Buddhism**, pretending to convey **divine will** — until my sons and I had converted.</v>
+        <v>Wine and glassware in candlelight — visual echo of the “altered drink” period described in Stage 1</v>
       </c>
       <c r="E48" t="str">
         <v/>
@@ -1514,16 +1514,16 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>founderStoryPage.phaseAStages[1].paragraphs[1]</v>
+        <v>founderStoryPage.phaseAStages[1].label</v>
       </c>
       <c r="B49" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C49" t="str">
-        <v>paragraph / other</v>
+        <v>label</v>
       </c>
       <c r="D49" t="str">
-        <v>It was a **grotesque joke**; we were **playthings**. Even so, we exchanged a great deal of **philosophical insight** during the deception.</v>
+        <v>A 2</v>
       </c>
       <c r="E49" t="str">
         <v/>
@@ -1537,16 +1537,16 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>founderStoryPage.phaseAStages[1].storylineClip.figureAlt</v>
+        <v>founderStoryPage.phaseAStages[1].stageTitle</v>
       </c>
       <c r="B50" t="str">
-        <v>创始人故事 / A 阶段 / 配图</v>
+        <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C50" t="str">
-        <v>label</v>
+        <v>heading</v>
       </c>
       <c r="D50" t="str">
-        <v>Golden Buddha statue — atmosphere of the religious theatre described in Stage 2</v>
+        <v>Cheating period 2</v>
       </c>
       <c r="E50" t="str">
         <v/>
@@ -1560,7 +1560,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>founderStoryPage.phaseAStages[2].label</v>
+        <v>founderStoryPage.phaseAStages[1].range</v>
       </c>
       <c r="B51" t="str">
         <v>创始人故事 / A 阶段</v>
@@ -1569,7 +1569,7 @@
         <v>label</v>
       </c>
       <c r="D51" t="str">
-        <v>A 3</v>
+        <v>July 2020 — 15 November 2020</v>
       </c>
       <c r="E51" t="str">
         <v/>
@@ -1583,16 +1583,16 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>founderStoryPage.phaseAStages[2].stageTitle</v>
+        <v>founderStoryPage.phaseAStages[1].paragraphs[0]</v>
       </c>
       <c r="B52" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C52" t="str">
-        <v>heading</v>
+        <v>paragraph / other</v>
       </c>
       <c r="D52" t="str">
-        <v>Exorcism period 1</v>
+        <v>During this interval, the low-level soul used **epilepsy-like seizures** to impersonate, in sequence, the **three greatest gods of Buddhism**, pretending to convey **divine will** — until my sons and I had converted.</v>
       </c>
       <c r="E52" t="str">
         <v/>
@@ -1606,16 +1606,16 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>founderStoryPage.phaseAStages[2].range</v>
+        <v>founderStoryPage.phaseAStages[1].paragraphs[1]</v>
       </c>
       <c r="B53" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C53" t="str">
-        <v>label</v>
+        <v>paragraph / other</v>
       </c>
       <c r="D53" t="str">
-        <v>15 November 2020 — July 2021</v>
+        <v>It was a **grotesque joke**; we were **playthings**. Even so, we exchanged a great deal of **philosophical insight** during the deception.</v>
       </c>
       <c r="E53" t="str">
         <v/>
@@ -1629,16 +1629,16 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>founderStoryPage.phaseAStages[2].paragraphs[0]</v>
+        <v>founderStoryPage.phaseAStages[1].storylineClip.figureAlt</v>
       </c>
       <c r="B54" t="str">
-        <v>创始人故事 / A 阶段</v>
+        <v>创始人故事 / A 阶段 / 配图</v>
       </c>
       <c r="C54" t="str">
-        <v>paragraph / other</v>
+        <v>label</v>
       </c>
       <c r="D54" t="str">
-        <v>On **15 November 2020**, the **true identities** of the souls inside us and their **tricks** were finally exposed. In fear and rage we tried to **exorcise** them.</v>
+        <v>Golden Buddha statue — atmosphere of the religious theatre described in Stage 2</v>
       </c>
       <c r="E54" t="str">
         <v/>
@@ -1652,16 +1652,16 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>founderStoryPage.phaseAStages[2].paragraphs[1]</v>
+        <v>founderStoryPage.phaseAStages[2].label</v>
       </c>
       <c r="B55" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C55" t="str">
-        <v>paragraph / other</v>
+        <v>label</v>
       </c>
       <c r="D55" t="str">
-        <v>Traditional methods failed repeatedly; we remembered they had always **forbidden** us to touch **strong magnets**. We began using magnets to **hurt** them.</v>
+        <v>A 3</v>
       </c>
       <c r="E55" t="str">
         <v/>
@@ -1675,16 +1675,16 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>founderStoryPage.phaseAStages[2].paragraphs[2]</v>
+        <v>founderStoryPage.phaseAStages[2].stageTitle</v>
       </c>
       <c r="B56" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C56" t="str">
-        <v>paragraph / other</v>
+        <v>heading</v>
       </c>
       <c r="D56" t="str">
-        <v>Within days the soul in my **elder son** could not endure it and **left first**; about **six weeks** later the soul in my **younger son** left for the same reason.</v>
+        <v>Exorcism period 1</v>
       </c>
       <c r="E56" t="str">
         <v/>
@@ -1698,16 +1698,16 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>founderStoryPage.phaseAStages[2].paragraphs[3]</v>
+        <v>founderStoryPage.phaseAStages[2].range</v>
       </c>
       <c r="B57" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C57" t="str">
-        <v>paragraph / other</v>
+        <v>label</v>
       </c>
       <c r="D57" t="str">
-        <v>The soul in **me** refused to depart even when injured. I found that a **strong electrostatic field** could severely weaken its discharging: my **epilepsy vanished** the moment that happened — yet the soul **remained inside**, playing hide-and-seek.</v>
+        <v>15 November 2020 — July 2021</v>
       </c>
       <c r="E57" t="str">
         <v/>
@@ -1721,16 +1721,16 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>founderStoryPage.phaseAStages[3].label</v>
+        <v>founderStoryPage.phaseAStages[2].paragraphs[0]</v>
       </c>
       <c r="B58" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C58" t="str">
-        <v>label</v>
+        <v>paragraph / other</v>
       </c>
       <c r="D58" t="str">
-        <v>A 4</v>
+        <v>On **15 November 2020**, the **true identities** of the souls inside us and their **tricks** were finally exposed. In fear and rage we tried to **exorcise** them.</v>
       </c>
       <c r="E58" t="str">
         <v/>
@@ -1744,16 +1744,16 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>founderStoryPage.phaseAStages[3].stageTitle</v>
+        <v>founderStoryPage.phaseAStages[2].paragraphs[1]</v>
       </c>
       <c r="B59" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C59" t="str">
-        <v>heading</v>
+        <v>paragraph / other</v>
       </c>
       <c r="D59" t="str">
-        <v>Exorcism period 2 · and high-level revealing</v>
+        <v>Traditional methods failed repeatedly; we remembered they had always **forbidden** us to touch **strong magnets**. We began using magnets to **hurt** them.</v>
       </c>
       <c r="E59" t="str">
         <v/>
@@ -1767,16 +1767,16 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>founderStoryPage.phaseAStages[3].range</v>
+        <v>founderStoryPage.phaseAStages[2].paragraphs[2]</v>
       </c>
       <c r="B60" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C60" t="str">
-        <v>label</v>
+        <v>paragraph / other</v>
       </c>
       <c r="D60" t="str">
-        <v>July 2021 — 4 April 2022</v>
+        <v>Within days the soul in my **elder son** could not endure it and **left first**; about **six weeks** later the soul in my **younger son** left for the same reason.</v>
       </c>
       <c r="E60" t="str">
         <v/>
@@ -1790,7 +1790,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>founderStoryPage.phaseAStages[3].paragraphs[0]</v>
+        <v>founderStoryPage.phaseAStages[2].paragraphs[3]</v>
       </c>
       <c r="B61" t="str">
         <v>创始人故事 / A 阶段</v>
@@ -1799,7 +1799,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D61" t="str">
-        <v>In this stage we **found and confirmed** several ways to interfere with, injure, and **kill ordinary souls**.</v>
+        <v>The soul in **me** refused to depart even when injured. I found that a **strong electrostatic field** could severely weaken its discharging: my **epilepsy vanished** the moment that happened — yet the soul **remained inside**, playing hide-and-seek.</v>
       </c>
       <c r="E61" t="str">
         <v/>
@@ -1813,16 +1813,16 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>founderStoryPage.phaseAStages[3].paragraphs[1]</v>
+        <v>founderStoryPage.phaseAStages[3].label</v>
       </c>
       <c r="B62" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C62" t="str">
-        <v>paragraph / other</v>
+        <v>label</v>
       </c>
       <c r="D62" t="str">
-        <v>The limits of **electrostatic and magnet** work drew the attention of a **high-level soul** who had died in China roughly **1,500 years ago**. It joined the exploration: **consciousness transmission** for hints, while **steering the ordinary soul’s behavior** until I learned how to kill and expel **precisely and efficiently**.</v>
+        <v>A 4</v>
       </c>
       <c r="E62" t="str">
         <v/>
@@ -1836,16 +1836,16 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>founderStoryPage.phaseAStages[3].paragraphs[2]</v>
+        <v>founderStoryPage.phaseAStages[3].stageTitle</v>
       </c>
       <c r="B63" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C63" t="str">
-        <v>paragraph / other</v>
+        <v>heading</v>
       </c>
       <c r="D63" t="str">
-        <v>Each day I **tangled, fought, and coexisted** with the ordinary soul — **enemy and ally** at once — and traded large amounts of **spirit-relevant knowledge**.</v>
+        <v>Exorcism period 2 · and high-level revealing</v>
       </c>
       <c r="E63" t="str">
         <v/>
@@ -1859,16 +1859,16 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>founderStoryPage.phaseAStages[3].paragraphs[3]</v>
+        <v>founderStoryPage.phaseAStages[3].range</v>
       </c>
       <c r="B64" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C64" t="str">
-        <v>paragraph / other</v>
+        <v>label</v>
       </c>
       <c r="D64" t="str">
-        <v>Finally the high-level soul **disclosed itself**, demonstrated **extraordinary abilities**, cleared up a year of confusion, taught me more of the **soul world** — then **left my body** and vanished quickly.</v>
+        <v>July 2021 — 4 April 2022</v>
       </c>
       <c r="E64" t="str">
         <v/>
@@ -1882,16 +1882,16 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>founderStoryPage.phaseAStages[4].label</v>
+        <v>founderStoryPage.phaseAStages[3].paragraphs[0]</v>
       </c>
       <c r="B65" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C65" t="str">
-        <v>label</v>
+        <v>paragraph / other</v>
       </c>
       <c r="D65" t="str">
-        <v>A 5</v>
+        <v>In this stage we **found and confirmed** several ways to interfere with, injure, and **kill ordinary souls**.</v>
       </c>
       <c r="E65" t="str">
         <v/>
@@ -1905,16 +1905,16 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>founderStoryPage.phaseAStages[4].stageTitle</v>
+        <v>founderStoryPage.phaseAStages[3].paragraphs[1]</v>
       </c>
       <c r="B66" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C66" t="str">
-        <v>heading</v>
+        <v>paragraph / other</v>
       </c>
       <c r="D66" t="str">
-        <v>Class-C2 Qing Xiaoxian · Class-C3 Qian Kai</v>
+        <v>The limits of **electrostatic and magnet** work drew the attention of a **high-level soul** who had died in China roughly **1,500 years ago**. It joined the exploration: **consciousness transmission** for hints, while **steering the ordinary soul’s behavior** until I learned how to kill and expel **precisely and efficiently**.</v>
       </c>
       <c r="E66" t="str">
         <v/>
@@ -1928,16 +1928,16 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>founderStoryPage.phaseAStages[4].range</v>
+        <v>founderStoryPage.phaseAStages[3].paragraphs[2]</v>
       </c>
       <c r="B67" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C67" t="str">
-        <v>label</v>
+        <v>paragraph / other</v>
       </c>
       <c r="D67" t="str">
-        <v>December 2023 — January 2025</v>
+        <v>Each day I **tangled, fought, and coexisted** with the ordinary soul — **enemy and ally** at once — and traded large amounts of **spirit-relevant knowledge**.</v>
       </c>
       <c r="E67" t="str">
         <v/>
@@ -1951,7 +1951,7 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>founderStoryPage.phaseAStages[4].paragraphs[0]</v>
+        <v>founderStoryPage.phaseAStages[3].paragraphs[3]</v>
       </c>
       <c r="B68" t="str">
         <v>创始人故事 / A 阶段</v>
@@ -1960,7 +1960,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D68" t="str">
-        <v>In **December 2023** I was again possessed by the **Class-C2** spirit **Qing Xiaoxian**. Across roughly **1,700 years** as a ghost it had devoured on the order of **5,000–10,000** other souls, becoming an **enormous entity**.</v>
+        <v>Finally the high-level soul **disclosed itself**, demonstrated **extraordinary abilities**, cleared up a year of confusion, taught me more of the **soul world** — then **left my body** and vanished quickly.</v>
       </c>
       <c r="E68" t="str">
         <v/>
@@ -1974,16 +1974,16 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>founderStoryPage.phaseAStages[4].paragraphs[1]</v>
+        <v>founderStoryPage.phaseAStages[4].label</v>
       </c>
       <c r="B69" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C69" t="str">
-        <v>paragraph / other</v>
+        <v>label</v>
       </c>
       <c r="D69" t="str">
-        <v>It turned the Woo home into a **haunted-house field**, spun **multiple avatars** onto both sons, and allowed its **core form** to coordinate those fragments **remotely**.</v>
+        <v>A 5</v>
       </c>
       <c r="E69" t="str">
         <v/>
@@ -1997,16 +1997,16 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>founderStoryPage.phaseAStages[4].paragraphs[2]</v>
+        <v>founderStoryPage.phaseAStages[4].stageTitle</v>
       </c>
       <c r="B70" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C70" t="str">
-        <v>paragraph / other</v>
+        <v>heading</v>
       </c>
       <c r="D70" t="str">
-        <v>In the father: **schizophrenia**, **bipolar disorder**, **epilepsy**, **somatization**, and **powerful electrical assaults** on the heart. In the sons: **fatigue (energy coupling)**, **depression**, **pain disorder**, **IBS**, and further somatic patterns.</v>
+        <v>Class-C2 Qing Xiaoxian · Class-C3 Qian Kai</v>
       </c>
       <c r="E70" t="str">
         <v/>
@@ -2020,16 +2020,16 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>founderStoryPage.phaseAStages[4].paragraphs[3]</v>
+        <v>founderStoryPage.phaseAStages[4].range</v>
       </c>
       <c r="B71" t="str">
         <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C71" t="str">
-        <v>paragraph / other</v>
+        <v>label</v>
       </c>
       <c r="D71" t="str">
-        <v>Father and sons continued to refine **exorcism** and **ghost-neutralization** until this entity was **fully destroyed**.</v>
+        <v>December 2023 — January 2025</v>
       </c>
       <c r="E71" t="str">
         <v/>
@@ -2043,7 +2043,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>founderStoryPage.phaseAStages[4].paragraphs[4]</v>
+        <v>founderStoryPage.phaseAStages[4].paragraphs[0]</v>
       </c>
       <c r="B72" t="str">
         <v>创始人故事 / A 阶段</v>
@@ -2052,7 +2052,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D72" t="str">
-        <v>From **September 2024** through **January 2025** I was possessed again by the **Class-C3** spirit **Qian Kai**. **Higher ghost density means greater power** — so Qian Kai **exceeded** Qing Xiaoxian in **thought-control** and **pathogenic force**. We continued **self-rescue** until this spirit, too, was **eliminated**.</v>
+        <v>In **December 2023** I was again possessed by the **Class-C2** spirit **Qing Xiaoxian**. Across roughly **1,700 years** as a ghost it had devoured on the order of **5,000–10,000** other souls, becoming an **enormous entity**.</v>
       </c>
       <c r="E72" t="str">
         <v/>
@@ -2066,16 +2066,16 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>founderStoryPage.phaseB.title</v>
+        <v>founderStoryPage.phaseAStages[4].paragraphs[1]</v>
       </c>
       <c r="B73" t="str">
-        <v>创始人故事 / Phase B</v>
+        <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C73" t="str">
-        <v>heading</v>
+        <v>paragraph / other</v>
       </c>
       <c r="D73" t="str">
-        <v>B阶段：2025年2月至2026年3月</v>
+        <v>It turned the Woo home into a **haunted-house field**, spun **multiple avatars** onto both sons, and allowed its **core form** to coordinate those fragments **remotely**.</v>
       </c>
       <c r="E73" t="str">
         <v/>
@@ -2089,16 +2089,16 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>founderStoryPage.phaseB.blocks[0].title</v>
+        <v>founderStoryPage.phaseAStages[4].paragraphs[2]</v>
       </c>
       <c r="B74" t="str">
-        <v>创始人故事 / Phase B</v>
+        <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C74" t="str">
-        <v>heading</v>
+        <v>paragraph / other</v>
       </c>
       <c r="D74" t="str">
-        <v>直播间规模与成就记录</v>
+        <v>In the father: **schizophrenia**, **bipolar disorder**, **epilepsy**, **somatization**, and **powerful electrical assaults** on the heart. In the sons: **fatigue (energy coupling)**, **depression**, **pain disorder**, **IBS**, and further somatic patterns.</v>
       </c>
       <c r="E74" t="str">
         <v/>
@@ -2112,16 +2112,16 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>founderStoryPage.phaseB.blocks[0].text</v>
+        <v>founderStoryPage.phaseAStages[4].paragraphs[3]</v>
       </c>
       <c r="B75" t="str">
-        <v>创始人故事 / Phase B</v>
+        <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C75" t="str">
         <v>paragraph / other</v>
       </c>
       <c r="D75" t="str">
-        <v>从 **2025年2月19日** 至 **12月24日**，**Caros** 在 **TikTok** 上总共进行了 **265 场直播**；在直播间取得了 **超凡的成就**。完整记录与链接见：{{%ACH%}}</v>
+        <v>Father and sons continued to refine **exorcism** and **ghost-neutralization** until this entity was **fully destroyed**.</v>
       </c>
       <c r="E75" t="str">
         <v/>
@@ -2135,16 +2135,16 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>founderStoryPage.phaseB.blocks[1].title</v>
+        <v>founderStoryPage.phaseAStages[4].paragraphs[4]</v>
       </c>
       <c r="B76" t="str">
-        <v>创始人故事 / Phase B</v>
+        <v>创始人故事 / A 阶段</v>
       </c>
       <c r="C76" t="str">
-        <v>heading</v>
+        <v>paragraph / other</v>
       </c>
       <c r="D76" t="str">
-        <v>Master Spirit、混合灵与远程能力</v>
+        <v>From **September 2024** through **January 2025** I was possessed again by the **Class-C3** spirit **Qian Kai**. **Higher ghost density means greater power** — so Qian Kai **exceeded** Qing Xiaoxian in **thought-control** and **pathogenic force**. We continued **self-rescue** until this spirit, too, was **eliminated**.</v>
       </c>
       <c r="E76" t="str">
         <v/>
@@ -2158,19 +2158,19 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>founderStoryPage.phaseB.blocks[1].text</v>
+        <v>founderStoryPage.phaseB.title</v>
       </c>
       <c r="B77" t="str">
         <v>创始人故事 / Phase B</v>
       </c>
       <c r="C77" t="str">
-        <v>paragraph / other</v>
+        <v>heading</v>
       </c>
       <c r="D77" t="str">
-        <v>大量的 **Master Spirit** 以及 **混合灵（hybrid spirit）** 与我们父子联系，让我们知道灵魂世界竟然有 **管理者** 与 **造物主** 层面的秩序。**Master Spirit** 给我们很多帮助与 **特别的超常力量**，使 **Caros** 在中国就可以 **远程制约** 远在地球另一端北美附体的鬼魂。</v>
+        <v/>
       </c>
       <c r="E77" t="str">
-        <v/>
+        <v>B阶段：2025年2月至2026年3月</v>
       </c>
       <c r="F77" t="str">
         <v/>
@@ -2181,7 +2181,7 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>founderStoryPage.phaseB.blocks[2].title</v>
+        <v>founderStoryPage.phaseB.blocks[0].title</v>
       </c>
       <c r="B78" t="str">
         <v>创始人故事 / Phase B</v>
@@ -2190,10 +2190,10 @@
         <v>heading</v>
       </c>
       <c r="D78" t="str">
-        <v>关于 A 阶段附体安排的说明</v>
+        <v/>
       </c>
       <c r="E78" t="str">
-        <v/>
+        <v>直播间规模与成就记录</v>
       </c>
       <c r="F78" t="str">
         <v/>
@@ -2204,7 +2204,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>founderStoryPage.phaseB.blocks[2].text</v>
+        <v>founderStoryPage.phaseB.blocks[0].text</v>
       </c>
       <c r="B79" t="str">
         <v>创始人故事 / Phase B</v>
@@ -2213,10 +2213,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D79" t="str">
-        <v>**最重要的是**，我们被告知：**A 阶段** 在我们身上附体的鬼魂都是被 **Master Spirit** **刻意安排** 进来的；这些附体之灵被清除是 **被许可作为研究使用** 的。</v>
+        <v/>
       </c>
       <c r="E79" t="str">
-        <v/>
+        <v>从 **2025年2月19日** 至 **12月24日**，**Caros** 在 **TikTok** 上总共进行了 **265 场直播**；在直播间取得了 **超凡的成就**。完整记录与链接见：{{%ACH%}}</v>
       </c>
       <c r="F79" t="str">
         <v/>
@@ -2227,7 +2227,7 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>founderStoryPage.phaseB.blocks[3].title</v>
+        <v>founderStoryPage.phaseB.blocks[1].title</v>
       </c>
       <c r="B80" t="str">
         <v>创始人故事 / Phase B</v>
@@ -2236,10 +2236,10 @@
         <v>heading</v>
       </c>
       <c r="D80" t="str">
-        <v>计划中的病痛与叙事</v>
+        <v/>
       </c>
       <c r="E80" t="str">
-        <v/>
+        <v>Master Spirit、混合灵与远程能力</v>
       </c>
       <c r="F80" t="str">
         <v/>
@@ -2250,7 +2250,7 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>founderStoryPage.phaseB.blocks[3].text</v>
+        <v>founderStoryPage.phaseB.blocks[1].text</v>
       </c>
       <c r="B81" t="str">
         <v>创始人故事 / Phase B</v>
@@ -2259,10 +2259,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D81" t="str">
-        <v>所有的 **病痛折磨**、**欺骗**、**戏弄性的故事** 也是他们计划的一部分，让我们了解其 **行事风格** 与 **性格秉性**。</v>
+        <v/>
       </c>
       <c r="E81" t="str">
-        <v/>
+        <v>大量的 **Master Spirit** 以及 **混合灵（hybrid spirit）** 与我们父子联系，让我们知道灵魂世界竟然有 **管理者** 与 **造物主** 层面的秩序。**Master Spirit** 给我们很多帮助与 **特别的超常力量**，使 **Caros** 在中国就可以 **远程制约** 远在地球另一端北美附体的鬼魂。</v>
       </c>
       <c r="F81" t="str">
         <v/>
@@ -2273,7 +2273,7 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>founderStoryPage.phaseB.blocks[4].title</v>
+        <v>founderStoryPage.phaseB.blocks[2].title</v>
       </c>
       <c r="B82" t="str">
         <v>创始人故事 / Phase B</v>
@@ -2282,10 +2282,10 @@
         <v>heading</v>
       </c>
       <c r="D82" t="str">
-        <v>对 Master Spirit 品性的认识</v>
+        <v/>
       </c>
       <c r="E82" t="str">
-        <v/>
+        <v>关于 A 阶段附体安排的说明</v>
       </c>
       <c r="F82" t="str">
         <v/>
@@ -2296,7 +2296,7 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>founderStoryPage.phaseB.blocks[4].text</v>
+        <v>founderStoryPage.phaseB.blocks[2].text</v>
       </c>
       <c r="B83" t="str">
         <v>创始人故事 / Phase B</v>
@@ -2305,10 +2305,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D83" t="str">
-        <v>这也让我们完整认识到：**Master Spirit** 并非像我们想象中的 **天使般的善良**；先前提供的帮助 **并非出于善良**，而是 **万有元神母体** 给他们安排的工作。大家可以通过 **A 阶段故事** 充分体会 **Master Spirit 团队的性格属性**。</v>
+        <v/>
       </c>
       <c r="E83" t="str">
-        <v/>
+        <v>**最重要的是**，我们被告知：**A 阶段** 在我们身上附体的鬼魂都是被 **Master Spirit** **刻意安排** 进来的；这些附体之灵被清除是 **被许可作为研究使用** 的。</v>
       </c>
       <c r="F83" t="str">
         <v/>
@@ -2319,7 +2319,7 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>founderStoryPage.phaseB.blocks[5].title</v>
+        <v>founderStoryPage.phaseB.blocks[3].title</v>
       </c>
       <c r="B84" t="str">
         <v>创始人故事 / Phase B</v>
@@ -2328,10 +2328,10 @@
         <v>heading</v>
       </c>
       <c r="D84" t="str">
-        <v>灵魂医学与影像档案</v>
+        <v/>
       </c>
       <c r="E84" t="str">
-        <v/>
+        <v>计划中的病痛与叙事</v>
       </c>
       <c r="F84" t="str">
         <v/>
@@ -2342,7 +2342,7 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>founderStoryPage.phaseB.blocks[5].text</v>
+        <v>founderStoryPage.phaseB.blocks[3].text</v>
       </c>
       <c r="B85" t="str">
         <v>创始人故事 / Phase B</v>
@@ -2351,10 +2351,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D85" t="str">
-        <v>在此期间，**正式创建了灵魂医学**；拍摄了 **《吴氏灵魂医学》** 与 **《万有元神母体》** 系列视频档案中的 **一部分视频**。</v>
+        <v/>
       </c>
       <c r="E85" t="str">
-        <v/>
+        <v>所有的 **病痛折磨**、**欺骗**、**戏弄性的故事** 也是他们计划的一部分，让我们了解其 **行事风格** 与 **性格秉性**。</v>
       </c>
       <c r="F85" t="str">
         <v/>
@@ -2365,19 +2365,19 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>founderTimeline[0].range</v>
+        <v>founderStoryPage.phaseB.blocks[4].title</v>
       </c>
       <c r="B86" t="str">
-        <v>创始人故事 / 年表</v>
+        <v>创始人故事 / Phase B</v>
       </c>
       <c r="C86" t="str">
-        <v>label</v>
+        <v>heading</v>
       </c>
       <c r="D86" t="str">
-        <v>May 2014 — Feb 2025</v>
+        <v/>
       </c>
       <c r="E86" t="str">
-        <v/>
+        <v>对 Master Spirit 品性的认识</v>
       </c>
       <c r="F86" t="str">
         <v/>
@@ -2388,19 +2388,19 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>founderTimeline[0].label</v>
+        <v>founderStoryPage.phaseB.blocks[4].text</v>
       </c>
       <c r="B87" t="str">
-        <v>创始人故事 / 年表</v>
+        <v>创始人故事 / Phase B</v>
       </c>
       <c r="C87" t="str">
-        <v>label</v>
+        <v>paragraph / other</v>
       </c>
       <c r="D87" t="str">
-        <v>Phase A — family field work</v>
+        <v/>
       </c>
       <c r="E87" t="str">
-        <v/>
+        <v>这也让我们完整认识到：**Master Spirit** 并非像我们想象中的 **天使般的善良**；先前提供的帮助 **并非出于善良**，而是 **万有元神母体** 给他们安排的工作。大家可以通过 **A 阶段故事** 充分体会 **Master Spirit 团队的性格属性**。</v>
       </c>
       <c r="F87" t="str">
         <v/>
@@ -2411,19 +2411,19 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>founderTimeline[1].range</v>
+        <v>founderStoryPage.phaseB.blocks[5].title</v>
       </c>
       <c r="B88" t="str">
-        <v>创始人故事 / 年表</v>
+        <v>创始人故事 / Phase B</v>
       </c>
       <c r="C88" t="str">
-        <v>label</v>
+        <v>heading</v>
       </c>
       <c r="D88" t="str">
-        <v>Mar 2018 — Jul 2020</v>
+        <v/>
       </c>
       <c r="E88" t="str">
-        <v/>
+        <v>灵魂医学与影像档案</v>
       </c>
       <c r="F88" t="str">
         <v/>
@@ -2434,19 +2434,19 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>founderTimeline[1].label</v>
+        <v>founderStoryPage.phaseB.blocks[5].text</v>
       </c>
       <c r="B89" t="str">
-        <v>创始人故事 / 年表</v>
+        <v>创始人故事 / Phase B</v>
       </c>
       <c r="C89" t="str">
-        <v>label</v>
+        <v>paragraph / other</v>
       </c>
       <c r="D89" t="str">
-        <v>Cheating Period 1</v>
+        <v/>
       </c>
       <c r="E89" t="str">
-        <v/>
+        <v>在此期间，**正式创建了灵魂医学**；拍摄了 **《吴氏灵魂医学》** 与 **《万有元神母体》** 系列视频档案中的 **一部分视频**。</v>
       </c>
       <c r="F89" t="str">
         <v/>
@@ -2457,7 +2457,7 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>founderTimeline[2].range</v>
+        <v>founderTimeline[0].range</v>
       </c>
       <c r="B90" t="str">
         <v>创始人故事 / 年表</v>
@@ -2466,7 +2466,7 @@
         <v>label</v>
       </c>
       <c r="D90" t="str">
-        <v>Jul 2020 — Nov 2020</v>
+        <v>May 2014 — Feb 2025</v>
       </c>
       <c r="E90" t="str">
         <v/>
@@ -2480,7 +2480,7 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>founderTimeline[2].label</v>
+        <v>founderTimeline[0].label</v>
       </c>
       <c r="B91" t="str">
         <v>创始人故事 / 年表</v>
@@ -2489,7 +2489,7 @@
         <v>label</v>
       </c>
       <c r="D91" t="str">
-        <v>Cheating period 2</v>
+        <v>Phase A — family field work</v>
       </c>
       <c r="E91" t="str">
         <v/>
@@ -2503,7 +2503,7 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>founderTimeline[3].range</v>
+        <v>founderTimeline[1].range</v>
       </c>
       <c r="B92" t="str">
         <v>创始人故事 / 年表</v>
@@ -2512,7 +2512,7 @@
         <v>label</v>
       </c>
       <c r="D92" t="str">
-        <v>Nov 2020 — Jul 2021</v>
+        <v>Mar 2018 — Jul 2020</v>
       </c>
       <c r="E92" t="str">
         <v/>
@@ -2526,7 +2526,7 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>founderTimeline[3].label</v>
+        <v>founderTimeline[1].label</v>
       </c>
       <c r="B93" t="str">
         <v>创始人故事 / 年表</v>
@@ -2535,7 +2535,7 @@
         <v>label</v>
       </c>
       <c r="D93" t="str">
-        <v>Exorcism period 1</v>
+        <v>Cheating Period 1</v>
       </c>
       <c r="E93" t="str">
         <v/>
@@ -2549,7 +2549,7 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>founderTimeline[4].range</v>
+        <v>founderTimeline[2].range</v>
       </c>
       <c r="B94" t="str">
         <v>创始人故事 / 年表</v>
@@ -2558,7 +2558,7 @@
         <v>label</v>
       </c>
       <c r="D94" t="str">
-        <v>Jul 2021 — Apr 2022</v>
+        <v>Jul 2020 — Nov 2020</v>
       </c>
       <c r="E94" t="str">
         <v/>
@@ -2572,7 +2572,7 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>founderTimeline[4].label</v>
+        <v>founderTimeline[2].label</v>
       </c>
       <c r="B95" t="str">
         <v>创始人故事 / 年表</v>
@@ -2581,7 +2581,7 @@
         <v>label</v>
       </c>
       <c r="D95" t="str">
-        <v>Exorcism 2 &amp; high-level revealing</v>
+        <v>Cheating period 2</v>
       </c>
       <c r="E95" t="str">
         <v/>
@@ -2595,7 +2595,7 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>founderTimeline[5].range</v>
+        <v>founderTimeline[3].range</v>
       </c>
       <c r="B96" t="str">
         <v>创始人故事 / 年表</v>
@@ -2604,7 +2604,7 @@
         <v>label</v>
       </c>
       <c r="D96" t="str">
-        <v>Dec 2023 — Jan 2025</v>
+        <v>Nov 2020 — Jul 2021</v>
       </c>
       <c r="E96" t="str">
         <v/>
@@ -2618,7 +2618,7 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>founderTimeline[5].label</v>
+        <v>founderTimeline[3].label</v>
       </c>
       <c r="B97" t="str">
         <v>创始人故事 / 年表</v>
@@ -2627,7 +2627,7 @@
         <v>label</v>
       </c>
       <c r="D97" t="str">
-        <v>Qing Xiaoxian (C2) · Qian Kai (C3)</v>
+        <v>Exorcism period 1</v>
       </c>
       <c r="E97" t="str">
         <v/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>founderTimeline[6].range</v>
+        <v>founderTimeline[4].range</v>
       </c>
       <c r="B98" t="str">
         <v>创始人故事 / 年表</v>
@@ -2650,7 +2650,7 @@
         <v>label</v>
       </c>
       <c r="D98" t="str">
-        <v>2025年2月—2026年3月</v>
+        <v>Jul 2021 — Apr 2022</v>
       </c>
       <c r="E98" t="str">
         <v/>
@@ -2664,7 +2664,7 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>founderTimeline[6].label</v>
+        <v>founderTimeline[4].label</v>
       </c>
       <c r="B99" t="str">
         <v>创始人故事 / 年表</v>
@@ -2673,7 +2673,7 @@
         <v>label</v>
       </c>
       <c r="D99" t="str">
-        <v>B阶段 · TikTok 直播与灵魂医学档案</v>
+        <v>Exorcism 2 &amp; high-level revealing</v>
       </c>
       <c r="E99" t="str">
         <v/>
@@ -2687,16 +2687,16 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>founderStoryIllustrations[0].alt</v>
+        <v>founderTimeline[5].range</v>
       </c>
       <c r="B100" t="str">
-        <v>创始人故事 / 插图说明</v>
+        <v>创始人故事 / 年表</v>
       </c>
       <c r="C100" t="str">
         <v>label</v>
       </c>
       <c r="D100" t="str">
-        <v>Night sky — doorway imagery</v>
+        <v>Dec 2023 — Jan 2025</v>
       </c>
       <c r="E100" t="str">
         <v/>
@@ -2710,16 +2710,16 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>founderStoryIllustrations[1].alt</v>
+        <v>founderTimeline[5].label</v>
       </c>
       <c r="B101" t="str">
-        <v>创始人故事 / 插图说明</v>
+        <v>创始人故事 / 年表</v>
       </c>
       <c r="C101" t="str">
         <v>label</v>
       </c>
       <c r="D101" t="str">
-        <v>Cosmos and emergence</v>
+        <v>Qing Xiaoxian (C2) · Qian Kai (C3)</v>
       </c>
       <c r="E101" t="str">
         <v/>
@@ -2733,19 +2733,19 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>founderStoryIllustrations[2].alt</v>
+        <v>founderTimeline[6].range</v>
       </c>
       <c r="B102" t="str">
-        <v>创始人故事 / 插图说明</v>
+        <v>创始人故事 / 年表</v>
       </c>
       <c r="C102" t="str">
         <v>label</v>
       </c>
       <c r="D102" t="str">
-        <v>Mountain dawn — long journey</v>
+        <v/>
       </c>
       <c r="E102" t="str">
-        <v/>
+        <v>2025年2月—2026年3月</v>
       </c>
       <c r="F102" t="str">
         <v/>
@@ -2756,19 +2756,19 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>founderStoryIllustrations[3].alt</v>
+        <v>founderTimeline[6].label</v>
       </c>
       <c r="B103" t="str">
-        <v>创始人故事 / 插图说明</v>
+        <v>创始人故事 / 年表</v>
       </c>
       <c r="C103" t="str">
         <v>label</v>
       </c>
       <c r="D103" t="str">
-        <v>Together — family path</v>
+        <v/>
       </c>
       <c r="E103" t="str">
-        <v/>
+        <v>B阶段 · TikTok 直播与灵魂医学档案</v>
       </c>
       <c r="F103" t="str">
         <v/>
@@ -2779,7 +2779,7 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>founderStoryIllustrations[4].alt</v>
+        <v>founderStoryIllustrations[0].alt</v>
       </c>
       <c r="B104" t="str">
         <v>创始人故事 / 插图说明</v>
@@ -2788,21 +2788,113 @@
         <v>label</v>
       </c>
       <c r="D104" t="str">
+        <v>Night sky — doorway imagery</v>
+      </c>
+      <c r="E104" t="str">
+        <v/>
+      </c>
+      <c r="F104" t="str">
+        <v/>
+      </c>
+      <c r="G104" t="str">
+        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>founderStoryIllustrations[1].alt</v>
+      </c>
+      <c r="B105" t="str">
+        <v>创始人故事 / 插图说明</v>
+      </c>
+      <c r="C105" t="str">
+        <v>label</v>
+      </c>
+      <c r="D105" t="str">
+        <v>Cosmos and emergence</v>
+      </c>
+      <c r="E105" t="str">
+        <v/>
+      </c>
+      <c r="F105" t="str">
+        <v/>
+      </c>
+      <c r="G105" t="str">
+        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>founderStoryIllustrations[2].alt</v>
+      </c>
+      <c r="B106" t="str">
+        <v>创始人故事 / 插图说明</v>
+      </c>
+      <c r="C106" t="str">
+        <v>label</v>
+      </c>
+      <c r="D106" t="str">
+        <v>Mountain dawn — long journey</v>
+      </c>
+      <c r="E106" t="str">
+        <v/>
+      </c>
+      <c r="F106" t="str">
+        <v/>
+      </c>
+      <c r="G106" t="str">
+        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>founderStoryIllustrations[3].alt</v>
+      </c>
+      <c r="B107" t="str">
+        <v>创始人故事 / 插图说明</v>
+      </c>
+      <c r="C107" t="str">
+        <v>label</v>
+      </c>
+      <c r="D107" t="str">
+        <v>Together — family path</v>
+      </c>
+      <c r="E107" t="str">
+        <v/>
+      </c>
+      <c r="F107" t="str">
+        <v/>
+      </c>
+      <c r="G107" t="str">
+        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>founderStoryIllustrations[4].alt</v>
+      </c>
+      <c r="B108" t="str">
+        <v>创始人故事 / 插图说明</v>
+      </c>
+      <c r="C108" t="str">
+        <v>label</v>
+      </c>
+      <c r="D108" t="str">
         <v>Broadcast and field</v>
       </c>
-      <c r="E104" t="str">
-        <v/>
-      </c>
-      <c r="F104" t="str">
-        <v/>
-      </c>
-      <c r="G104" t="str">
+      <c r="E108" t="str">
+        <v/>
+      </c>
+      <c r="F108" t="str">
+        <v/>
+      </c>
+      <c r="G108" t="str">
         <v>founderStory2026Content.ts — ** in source = emphasis</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G104"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G108"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(founder-story): Phase B EN source in content, Chinese in zh.i18n; localized achievements link
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/page-copy/03-创始人故事.xlsx
+++ b/docs/page-copy/03-创始人故事.xlsx
@@ -433,7 +433,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>founderStory.collapsePhaseA</v>
+        <v>founderStory.achievementsFeaturePageLink</v>
       </c>
       <c r="B2" t="str">
         <v>创始人故事 / i18n</v>
@@ -442,10 +442,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D2" t="str">
-        <v>✦  Hide Phase A detail  ▲</v>
+        <v>2025 Livestream Achievements</v>
       </c>
       <c r="E2" t="str">
-        <v>✦  收起 A 阶段详情  ▲</v>
+        <v>《2025直播间成就》专题页</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -456,7 +456,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>founderStory.collapsePhaseB</v>
+        <v>founderStory.collapsePhaseA</v>
       </c>
       <c r="B3" t="str">
         <v>创始人故事 / i18n</v>
@@ -465,10 +465,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D3" t="str">
-        <v>✦  Hide Phase B detail  ▲</v>
+        <v>✦  Hide Phase A detail  ▲</v>
       </c>
       <c r="E3" t="str">
-        <v>✦  收起 B 阶段详情  ▲</v>
+        <v>✦  收起 A 阶段详情  ▲</v>
       </c>
       <c r="F3" t="str">
         <v/>
@@ -479,7 +479,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>founderStory.expandPhaseA</v>
+        <v>founderStory.collapsePhaseB</v>
       </c>
       <c r="B4" t="str">
         <v>创始人故事 / i18n</v>
@@ -488,10 +488,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D4" t="str">
-        <v>✦  Show Phase A chronology &amp; full detail  ▼</v>
+        <v>✦  Hide Phase B detail  ▲</v>
       </c>
       <c r="E4" t="str">
-        <v>✦  展开 A 阶段年表与完整叙事  ▼</v>
+        <v>✦  收起 B 阶段详情  ▲</v>
       </c>
       <c r="F4" t="str">
         <v/>
@@ -502,7 +502,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>founderStory.expandPhaseB</v>
+        <v>founderStory.expandPhaseA</v>
       </c>
       <c r="B5" t="str">
         <v>创始人故事 / i18n</v>
@@ -511,10 +511,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D5" t="str">
-        <v>✦  Show Phase B chronology &amp; full detail  ▼</v>
+        <v>✦  Show Phase A chronology &amp; full detail  ▼</v>
       </c>
       <c r="E5" t="str">
-        <v>✦  展开 B 阶段年表与完整叙事  ▼</v>
+        <v>✦  展开 A 阶段年表与完整叙事  ▼</v>
       </c>
       <c r="F5" t="str">
         <v/>
@@ -525,7 +525,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>founderStory.phaseAUmbrellaCaption</v>
+        <v>founderStory.expandPhaseB</v>
       </c>
       <c r="B6" t="str">
         <v>创始人故事 / i18n</v>
@@ -534,10 +534,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D6" t="str">
-        <v>Overall window for family field work (Phase A). Sub-stages A1–A5 below: date line first, then narrative.</v>
+        <v>✦  Show Phase B chronology &amp; full detail  ▼</v>
       </c>
       <c r="E6" t="str">
-        <v>A 阶段总览时间窗（家庭田野）。以下 A1–A5：每条先时间线，再正文，仅保留小节标题 A1、A2…</v>
+        <v>✦  展开 B 阶段年表与完整叙事  ▼</v>
       </c>
       <c r="F6" t="str">
         <v/>
@@ -548,7 +548,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>founderStory.storylineClipLead</v>
+        <v>founderStory.phaseAUmbrellaCaption</v>
       </c>
       <c r="B7" t="str">
         <v>创始人故事 / i18n</v>
@@ -557,10 +557,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D7" t="str">
-        <v>**Stage {{stage}}** on the original storyline: companion image plus the same YouTube session (embedded below). For context see</v>
+        <v>Overall window for family field work (Phase A). Sub-stages A1–A5 below: date line first, then narrative.</v>
       </c>
       <c r="E7" t="str">
-        <v>与旧站叙事 **第 {{stage}} 阶段**对应：配图 + 同一则 YouTube（下方嵌入）。完整语境见</v>
+        <v>A 阶段总览时间窗（家庭田野）。以下 A1–A5：每条先时间线，再正文，仅保留小节标题 A1、A2…</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -571,7 +571,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>founderStory.storylineClipPageLink</v>
+        <v>founderStory.storylineClipLead</v>
       </c>
       <c r="B8" t="str">
         <v>创始人故事 / i18n</v>
@@ -580,10 +580,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D8" t="str">
-        <v>Storyline of Woos</v>
+        <v>**Stage {{stage}}** on the original storyline: companion image plus the same YouTube session (embedded below). For context see</v>
       </c>
       <c r="E8" t="str">
-        <v>《Storyline of Woos》</v>
+        <v>与旧站叙事 **第 {{stage}} 阶段**对应：配图 + 同一则 YouTube（下方嵌入）。完整语境见</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -594,19 +594,19 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>founderStory.storylineYoutubeIframeTitle</v>
+        <v>founderStory.storylineClipPageLink</v>
       </c>
       <c r="B9" t="str">
         <v>创始人故事 / i18n</v>
       </c>
       <c r="C9" t="str">
-        <v>heading</v>
+        <v>paragraph / other</v>
       </c>
       <c r="D9" t="str">
-        <v>Storyline of Woos — Stage {{stage}} recording</v>
+        <v>Storyline of Woos</v>
       </c>
       <c r="E9" t="str">
-        <v>Storyline of Woos — 第 {{stage}} 阶段录像</v>
+        <v>《Storyline of Woos》</v>
       </c>
       <c r="F9" t="str">
         <v/>
@@ -617,39 +617,39 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>founderStorySurfaceCopy.heroNamesLine</v>
+        <v>founderStory.storylineYoutubeIframeTitle</v>
       </c>
       <c r="B10" t="str">
-        <v>创始人故事 / 英雄区副标题</v>
+        <v>创始人故事 / i18n</v>
       </c>
       <c r="C10" t="str">
-        <v>label</v>
+        <v>heading</v>
       </c>
       <c r="D10" t="str">
-        <v>John Long Woo · Caros · Sam</v>
+        <v>Storyline of Woos — Stage {{stage}} recording</v>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>Storyline of Woos — 第 {{stage}} 阶段录像</v>
       </c>
       <c r="F10" t="str">
         <v/>
       </c>
       <c r="G10" t="str">
-        <v>founderStorySurfaceCopy — FounderStoryView chrome</v>
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>founderStorySurfaceCopy.backToAbout</v>
+        <v>founderStorySurfaceCopy.heroNamesLine</v>
       </c>
       <c r="B11" t="str">
-        <v>创始人故事 / 返回</v>
+        <v>创始人故事 / 英雄区副标题</v>
       </c>
       <c r="C11" t="str">
-        <v>button / link</v>
+        <v>label</v>
       </c>
       <c r="D11" t="str">
-        <v>← Organization overview</v>
+        <v>John Long Woo · Caros · Sam</v>
       </c>
       <c r="E11" t="str">
         <v/>
@@ -663,16 +663,16 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>founderStorySurfaceCopy.legacyTimelineLink</v>
+        <v>founderStorySurfaceCopy.backToAbout</v>
       </c>
       <c r="B12" t="str">
-        <v>创始人故事 / 页脚外链</v>
+        <v>创始人故事 / 返回</v>
       </c>
       <c r="C12" t="str">
         <v>button / link</v>
       </c>
       <c r="D12" t="str">
-        <v>Earlier staged timeline on the legacy site</v>
+        <v>← Organization overview</v>
       </c>
       <c r="E12" t="str">
         <v/>
@@ -686,19 +686,19 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>founderStorySurfaceCopy.achievementsFeaturePageLink</v>
+        <v>founderStorySurfaceCopy.legacyTimelineLink</v>
       </c>
       <c r="B13" t="str">
-        <v>创始人故事 / Phase B 内链（替换 {{%ACH%}}）</v>
+        <v>创始人故事 / 页脚外链</v>
       </c>
       <c r="C13" t="str">
         <v>button / link</v>
       </c>
       <c r="D13" t="str">
-        <v/>
+        <v>Earlier staged timeline on the legacy site</v>
       </c>
       <c r="E13" t="str">
-        <v>《2025直播间成就》专题页</v>
+        <v/>
       </c>
       <c r="F13" t="str">
         <v/>
@@ -2167,7 +2167,7 @@
         <v>heading</v>
       </c>
       <c r="D77" t="str">
-        <v/>
+        <v>Phase B — February 2025 through March 2026</v>
       </c>
       <c r="E77" t="str">
         <v>B阶段：2025年2月至2026年3月</v>
@@ -2176,7 +2176,7 @@
         <v/>
       </c>
       <c r="G77" t="str">
-        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+        <v>Phase B: EN = content file; 中文 = zh.ts → founderStory.phaseB.title</v>
       </c>
     </row>
     <row r="78">
@@ -2190,7 +2190,7 @@
         <v>heading</v>
       </c>
       <c r="D78" t="str">
-        <v/>
+        <v>Livestream scale and documented outcomes</v>
       </c>
       <c r="E78" t="str">
         <v>直播间规模与成就记录</v>
@@ -2199,7 +2199,7 @@
         <v/>
       </c>
       <c r="G78" t="str">
-        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+        <v>Phase B: EN = content file; 中文 = zh.ts → founderStory.phaseB.block0.title</v>
       </c>
     </row>
     <row r="79">
@@ -2213,7 +2213,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D79" t="str">
-        <v/>
+        <v>From **19 February 2025** through **24 December 2025**, **Caros** hosted **265** sessions on **TikTok Live** and achieved **extraordinary outcomes** in the broadcast field. Full documentation and links: {{%ACH%}}</v>
       </c>
       <c r="E79" t="str">
         <v>从 **2025年2月19日** 至 **12月24日**，**Caros** 在 **TikTok** 上总共进行了 **265 场直播**；在直播间取得了 **超凡的成就**。完整记录与链接见：{{%ACH%}}</v>
@@ -2222,7 +2222,7 @@
         <v/>
       </c>
       <c r="G79" t="str">
-        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+        <v>Phase B: EN = content file; 中文 = zh.ts → founderStory.phaseB.block0.text</v>
       </c>
     </row>
     <row r="80">
@@ -2236,7 +2236,7 @@
         <v>heading</v>
       </c>
       <c r="D80" t="str">
-        <v/>
+        <v>Master Spirits, hybrid spirits, and remote capacity</v>
       </c>
       <c r="E80" t="str">
         <v>Master Spirit、混合灵与远程能力</v>
@@ -2245,7 +2245,7 @@
         <v/>
       </c>
       <c r="G80" t="str">
-        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+        <v>Phase B: EN = content file; 中文 = zh.ts → founderStory.phaseB.block1.title</v>
       </c>
     </row>
     <row r="81">
@@ -2259,7 +2259,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D81" t="str">
-        <v/>
+        <v>A great many **Master Spirits** and **hybrid spirits** reached out to us as father and sons, revealing that the spirit world includes order at the levels of **administrators** and **creator-class** structure. **Master Spirits** gave us extensive support and **unusual abilities**, so that **Caros**, **while in China**, could **remotely regulate** attached spirits on **hosts in North America** on the far side of the globe.</v>
       </c>
       <c r="E81" t="str">
         <v>大量的 **Master Spirit** 以及 **混合灵（hybrid spirit）** 与我们父子联系，让我们知道灵魂世界竟然有 **管理者** 与 **造物主** 层面的秩序。**Master Spirit** 给我们很多帮助与 **特别的超常力量**，使 **Caros** 在中国就可以 **远程制约** 远在地球另一端北美附体的鬼魂。</v>
@@ -2268,7 +2268,7 @@
         <v/>
       </c>
       <c r="G81" t="str">
-        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+        <v>Phase B: EN = content file; 中文 = zh.ts → founderStory.phaseB.block1.text</v>
       </c>
     </row>
     <row r="82">
@@ -2282,7 +2282,7 @@
         <v>heading</v>
       </c>
       <c r="D82" t="str">
-        <v/>
+        <v>How Phase A attachments were arranged</v>
       </c>
       <c r="E82" t="str">
         <v>关于 A 阶段附体安排的说明</v>
@@ -2291,7 +2291,7 @@
         <v/>
       </c>
       <c r="G82" t="str">
-        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+        <v>Phase B: EN = content file; 中文 = zh.ts → founderStory.phaseB.block2.title</v>
       </c>
     </row>
     <row r="83">
@@ -2305,7 +2305,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D83" t="str">
-        <v/>
+        <v>**Most importantly**, we were told: every attached spirit on us during **Phase A** was **deliberately placed** by **Master Spirits**; clearing those presences was **authorized to serve as research material**.</v>
       </c>
       <c r="E83" t="str">
         <v>**最重要的是**，我们被告知：**A 阶段** 在我们身上附体的鬼魂都是被 **Master Spirit** **刻意安排** 进来的；这些附体之灵被清除是 **被许可作为研究使用** 的。</v>
@@ -2314,7 +2314,7 @@
         <v/>
       </c>
       <c r="G83" t="str">
-        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+        <v>Phase B: EN = content file; 中文 = zh.ts → founderStory.phaseB.block2.text</v>
       </c>
     </row>
     <row r="84">
@@ -2328,7 +2328,7 @@
         <v>heading</v>
       </c>
       <c r="D84" t="str">
-        <v/>
+        <v>Illness, deception, and narrative as part of the plan</v>
       </c>
       <c r="E84" t="str">
         <v>计划中的病痛与叙事</v>
@@ -2337,7 +2337,7 @@
         <v/>
       </c>
       <c r="G84" t="str">
-        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+        <v>Phase B: EN = content file; 中文 = zh.ts → founderStory.phaseB.block3.title</v>
       </c>
     </row>
     <row r="85">
@@ -2351,7 +2351,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D85" t="str">
-        <v/>
+        <v>The **suffering**, **deception**, and **taunting storylines** were also part of their plan—so we could learn their **operating style** and **disposition**.</v>
       </c>
       <c r="E85" t="str">
         <v>所有的 **病痛折磨**、**欺骗**、**戏弄性的故事** 也是他们计划的一部分，让我们了解其 **行事风格** 与 **性格秉性**。</v>
@@ -2360,7 +2360,7 @@
         <v/>
       </c>
       <c r="G85" t="str">
-        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+        <v>Phase B: EN = content file; 中文 = zh.ts → founderStory.phaseB.block3.text</v>
       </c>
     </row>
     <row r="86">
@@ -2374,7 +2374,7 @@
         <v>heading</v>
       </c>
       <c r="D86" t="str">
-        <v/>
+        <v>Understanding Master Spirit character</v>
       </c>
       <c r="E86" t="str">
         <v>对 Master Spirit 品性的认识</v>
@@ -2383,7 +2383,7 @@
         <v/>
       </c>
       <c r="G86" t="str">
-        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+        <v>Phase B: EN = content file; 中文 = zh.ts → founderStory.phaseB.block4.title</v>
       </c>
     </row>
     <row r="87">
@@ -2397,7 +2397,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D87" t="str">
-        <v/>
+        <v>That also showed us clearly: **Master Spirits** are **not** **angel-good** in the way we imagined; the help offered earlier was **not** driven by **kindness** but by **assignments** from the **Universal Matrix of Meta Awareness**. The **Phase A** stories convey the **temperament of the Master Spirit team** in depth.</v>
       </c>
       <c r="E87" t="str">
         <v>这也让我们完整认识到：**Master Spirit** 并非像我们想象中的 **天使般的善良**；先前提供的帮助 **并非出于善良**，而是 **万有元神母体** 给他们安排的工作。大家可以通过 **A 阶段故事** 充分体会 **Master Spirit 团队的性格属性**。</v>
@@ -2406,7 +2406,7 @@
         <v/>
       </c>
       <c r="G87" t="str">
-        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+        <v>Phase B: EN = content file; 中文 = zh.ts → founderStory.phaseB.block4.text</v>
       </c>
     </row>
     <row r="88">
@@ -2420,7 +2420,7 @@
         <v>heading</v>
       </c>
       <c r="D88" t="str">
-        <v/>
+        <v>Spirit Medicine and video archives</v>
       </c>
       <c r="E88" t="str">
         <v>灵魂医学与影像档案</v>
@@ -2429,7 +2429,7 @@
         <v/>
       </c>
       <c r="G88" t="str">
-        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+        <v>Phase B: EN = content file; 中文 = zh.ts → founderStory.phaseB.block5.title</v>
       </c>
     </row>
     <row r="89">
@@ -2443,7 +2443,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D89" t="str">
-        <v/>
+        <v>During this period **Spirit Medicine was formally established**; we produced **part of** the **Woos Spirit Medicine** and **Universal Matrix of Meta Awareness** video archives.</v>
       </c>
       <c r="E89" t="str">
         <v>在此期间，**正式创建了灵魂医学**；拍摄了 **《吴氏灵魂医学》** 与 **《万有元神母体》** 系列视频档案中的 **一部分视频**。</v>
@@ -2452,7 +2452,7 @@
         <v/>
       </c>
       <c r="G89" t="str">
-        <v>founderStory2026Content.ts — ** in source = emphasis</v>
+        <v>Phase B: EN = content file; 中文 = zh.ts → founderStory.phaseB.block5.text</v>
       </c>
     </row>
     <row r="90">

</xml_diff>

<commit_message>
Sync: founder story xlsx edits and regenerated page copy
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/page-copy/03-创始人故事.xlsx
+++ b/docs/page-copy/03-创始人故事.xlsx
@@ -1680,10 +1680,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D56" t="str">
-        <v>In this phase, Caros Woo communicated with a large number of attached **spirits (ghosts)** in North America through TikTok live streams, completely confirming all the spirit world truths we obtained in Phase A. With the help of master spirits, Caros Woo obtained the superpower to remotely control attached **spirits (ghosts)** in North America. This superpower is the foundation upon which we built ASRA.</v>
+        <v xml:space="preserve">In this phase, Caros Woo communicated with a large number of attached **spirits (ghosts)** in North America through TikTok live streams, completely confirming all the spirit world truths we obtained in Phase A. </v>
       </c>
       <c r="E56" t="str">
-        <v>在这个阶段，Caros Woo通过TikTok直播间与北美的大量附体鬼魂进行了交流，完全证实了A阶段我们获得的所有灵魂世界真相。并且在高级控制灵的帮助下，Caros Woo获得了远程控制北美附体鬼魂的超能力。这种超能力正是我们建设ASRA的基础。</v>
+        <v>在这个阶段，Caros Woo通过TikTok直播间与北美的大量附体鬼魂进行了交流，完全证实了A阶段我们获得的所有灵魂世界真相。</v>
       </c>
       <c r="F56" t="str">
         <v/>

</xml_diff>